<commit_message>
finish role playing evaluaiton code
</commit_message>
<xml_diff>
--- a/data/de-escalation training dataset.xlsx
+++ b/data/de-escalation training dataset.xlsx
@@ -1,23 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10830"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mdhasebulhasan/Documents/Research/de-escaltion/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B889595D-1478-CE49-9819-A8D70B26B9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="synthesis_dataset"/>
-    <sheet r:id="rId2" sheetId="2" name="Data_with_negative_example"/>
-    <sheet r:id="rId3" sheetId="3" name="de_escalation_evaluation"/>
-    <sheet r:id="rId4" sheetId="4" name="role_playing_evaluation"/>
+    <sheet name="synthesis_dataset" sheetId="1" r:id="rId1"/>
+    <sheet name="Data_with_negative_example" sheetId="2" r:id="rId2"/>
+    <sheet name="de_escalation_evaluation" sheetId="3" r:id="rId3"/>
+    <sheet name="role_playing_evaluation" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="131">
   <si>
     <t>Conversation_Id</t>
   </si>
@@ -1838,12 +1857,14 @@
 •	He is unarmed.
 </t>
   </si>
+  <si>
+    <t>ID</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1860,7 +1881,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1892,59 +1913,50 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1955,10 +1967,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
@@ -1996,71 +2008,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -2088,7 +2100,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -2111,11 +2123,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -2124,13 +2136,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -2140,7 +2152,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -2149,7 +2161,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2158,7 +2170,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2166,10 +2178,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -2234,29 +2246,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:M37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" style="13" width="14.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="13" width="14.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="14" width="31.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="14" width="27.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="14" width="60.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="14" width="37.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="14" width="28.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="14" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="13" width="17.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="14" width="102.57642857142856" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="11" width="28.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="11" width="87.14785714285713" customWidth="1" bestFit="1"/>
+    <col min="1" max="2" width="14.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.5" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.5" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="60.5" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="37.1640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" style="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.1640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="102.5" style="9" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="87.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>38</v>
       </c>
@@ -2297,7 +2308,7 @@
         <v>99</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="669">
+    <row r="2" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -2336,7 +2347,7 @@
       </c>
       <c r="M2" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="282">
+    <row r="3" spans="1:13" ht="282" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -2375,7 +2386,7 @@
       </c>
       <c r="M3" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="234">
+    <row r="4" spans="1:13" ht="234" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -2412,9 +2423,8 @@
       <c r="L4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M4" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="690">
+    </row>
+    <row r="5" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -2451,9 +2461,8 @@
       <c r="L5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="M5" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="618">
+    </row>
+    <row r="6" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -2490,9 +2499,8 @@
       <c r="L6" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="M6" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="426">
+    </row>
+    <row r="7" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -2529,9 +2537,8 @@
       <c r="L7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="M7" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="474">
+    </row>
+    <row r="8" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -2568,9 +2575,8 @@
       <c r="L8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M8" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="642">
+    </row>
+    <row r="9" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -2607,9 +2613,8 @@
       <c r="L9" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="M9" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="330">
+    </row>
+    <row r="10" spans="1:13" ht="330" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -2646,9 +2651,8 @@
       <c r="L10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="M10" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="786">
+    </row>
+    <row r="11" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -2685,9 +2689,8 @@
       <c r="L11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="M11" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="690">
+    </row>
+    <row r="12" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -2724,11 +2727,10 @@
       <c r="L12" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="M12" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="378">
+    </row>
+    <row r="13" spans="1:13" ht="378" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5">
-        <f>A12+1</f>
+        <v>12</v>
       </c>
       <c r="B13" s="5">
         <v>2</v>
@@ -2763,11 +2765,10 @@
       <c r="L13" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="M13" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="450">
+    </row>
+    <row r="14" spans="1:13" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="5">
-        <f>A13+1</f>
+        <v>13</v>
       </c>
       <c r="B14" s="5">
         <v>3</v>
@@ -2802,11 +2803,10 @@
       <c r="L14" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="M14" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="402">
+    </row>
+    <row r="15" spans="1:13" ht="402" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5">
-        <f>A14+1</f>
+        <v>14</v>
       </c>
       <c r="B15" s="5">
         <v>3</v>
@@ -2841,11 +2841,10 @@
       <c r="L15" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="M15" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="306">
+    </row>
+    <row r="16" spans="1:13" ht="306" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="5">
-        <f>A15+1</f>
+        <v>15</v>
       </c>
       <c r="B16" s="5">
         <v>3</v>
@@ -2880,11 +2879,10 @@
       <c r="L16" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="M16" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="546">
+    </row>
+    <row r="17" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="5">
-        <f>A16+1</f>
+        <v>16</v>
       </c>
       <c r="B17" s="5">
         <v>3</v>
@@ -2919,11 +2917,10 @@
       <c r="L17" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="M17" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="702">
+    </row>
+    <row r="18" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="5">
-        <f>A17+1</f>
+        <v>17</v>
       </c>
       <c r="B18" s="5">
         <v>3</v>
@@ -2958,11 +2955,10 @@
       <c r="L18" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="M18" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="426">
+    </row>
+    <row r="19" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="5">
-        <f>A18+1</f>
+        <v>18</v>
       </c>
       <c r="B19" s="5">
         <v>3</v>
@@ -2997,11 +2993,10 @@
       <c r="L19" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="M19" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="330">
+    </row>
+    <row r="20" spans="1:12" ht="330" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="5">
-        <f>A19+1</f>
+        <v>19</v>
       </c>
       <c r="B20" s="5">
         <v>4</v>
@@ -3036,11 +3031,10 @@
       <c r="L20" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M20" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="306">
+    </row>
+    <row r="21" spans="1:12" ht="306" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5">
-        <f>A20+1</f>
+        <v>20</v>
       </c>
       <c r="B21" s="5">
         <v>4</v>
@@ -3075,11 +3069,10 @@
       <c r="L21" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M21" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="258">
+    </row>
+    <row r="22" spans="1:12" ht="258" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="5">
-        <f>A21+1</f>
+        <v>21</v>
       </c>
       <c r="B22" s="5">
         <v>4</v>
@@ -3114,11 +3107,10 @@
       <c r="L22" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M22" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="546">
+    </row>
+    <row r="23" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="5">
-        <f>A22+1</f>
+        <v>22</v>
       </c>
       <c r="B23" s="5">
         <v>4</v>
@@ -3153,11 +3145,10 @@
       <c r="L23" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="M23" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="498">
+    </row>
+    <row r="24" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="5">
-        <f>A23+1</f>
+        <v>23</v>
       </c>
       <c r="B24" s="5">
         <v>4</v>
@@ -3192,11 +3183,10 @@
       <c r="L24" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="M24" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="426">
+    </row>
+    <row r="25" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="5">
-        <f>A24+1</f>
+        <v>24</v>
       </c>
       <c r="B25" s="5">
         <v>4</v>
@@ -3231,11 +3221,10 @@
       <c r="L25" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="M25" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="402">
+    </row>
+    <row r="26" spans="1:12" ht="402" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="5">
-        <f>A25+1</f>
+        <v>25</v>
       </c>
       <c r="B26" s="5">
         <v>5</v>
@@ -3270,11 +3259,10 @@
       <c r="L26" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M26" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="306">
+    </row>
+    <row r="27" spans="1:12" ht="306" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="5">
-        <f>A26+1</f>
+        <v>26</v>
       </c>
       <c r="B27" s="5">
         <v>5</v>
@@ -3309,11 +3297,10 @@
       <c r="L27" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M27" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="258">
+    </row>
+    <row r="28" spans="1:12" ht="258" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="5">
-        <f>A27+1</f>
+        <v>27</v>
       </c>
       <c r="B28" s="5">
         <v>5</v>
@@ -3348,11 +3335,10 @@
       <c r="L28" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M28" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="594">
+    </row>
+    <row r="29" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="5">
-        <f>A28+1</f>
+        <v>28</v>
       </c>
       <c r="B29" s="5">
         <v>5</v>
@@ -3387,11 +3373,10 @@
       <c r="L29" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="M29" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="546">
+    </row>
+    <row r="30" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="5">
-        <f>A29+1</f>
+        <v>29</v>
       </c>
       <c r="B30" s="5">
         <v>5</v>
@@ -3426,11 +3411,10 @@
       <c r="L30" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="M30" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="426">
+    </row>
+    <row r="31" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="5">
-        <f>A30+1</f>
+        <v>30</v>
       </c>
       <c r="B31" s="5">
         <v>5</v>
@@ -3465,12 +3449,9 @@
       <c r="L31" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="M31" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="5">
-        <f>A31+1</f>
-      </c>
+    </row>
+    <row r="32" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="5"/>
       <c r="B32" s="5"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
@@ -3480,14 +3461,9 @@
       <c r="H32" s="6"/>
       <c r="I32" s="5"/>
       <c r="J32" s="2"/>
-      <c r="K32" s="8"/>
-      <c r="L32" s="8"/>
-      <c r="M32" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="5">
-        <f>A32+1</f>
-      </c>
+    </row>
+    <row r="33" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="5"/>
       <c r="B33" s="5"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
@@ -3497,14 +3473,9 @@
       <c r="H33" s="6"/>
       <c r="I33" s="5"/>
       <c r="J33" s="6"/>
-      <c r="K33" s="8"/>
-      <c r="L33" s="8"/>
-      <c r="M33" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="5">
-        <f>A33+1</f>
-      </c>
+    </row>
+    <row r="34" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="5"/>
       <c r="B34" s="5"/>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
@@ -3514,14 +3485,9 @@
       <c r="H34" s="6"/>
       <c r="I34" s="5"/>
       <c r="J34" s="6"/>
-      <c r="K34" s="8"/>
-      <c r="L34" s="8"/>
-      <c r="M34" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
-      <c r="A35" s="5">
-        <f>A34+1</f>
-      </c>
+    </row>
+    <row r="35" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="5"/>
       <c r="B35" s="5"/>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
@@ -3531,14 +3497,9 @@
       <c r="H35" s="6"/>
       <c r="I35" s="5"/>
       <c r="J35" s="6"/>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="5">
-        <f>A35+1</f>
-      </c>
+    </row>
+    <row r="36" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="5"/>
       <c r="B36" s="5"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
@@ -3548,14 +3509,9 @@
       <c r="H36" s="6"/>
       <c r="I36" s="5"/>
       <c r="J36" s="6"/>
-      <c r="K36" s="8"/>
-      <c r="L36" s="8"/>
-      <c r="M36" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="5">
-        <f>A36+1</f>
-      </c>
+    </row>
+    <row r="37" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="5"/>
       <c r="B37" s="5"/>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
@@ -3565,9 +3521,6 @@
       <c r="H37" s="6"/>
       <c r="I37" s="5"/>
       <c r="J37" s="6"/>
-      <c r="K37" s="8"/>
-      <c r="L37" s="8"/>
-      <c r="M37" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3575,29 +3528,28 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F102"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" style="10" width="22.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="11" width="31.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="11" width="32.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="22.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.5" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B1" s="6" t="s">
+    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -3610,11 +3562,11 @@
         <v>41</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="5">
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -3626,15 +3578,15 @@
       <c r="E2" s="1">
         <v>1</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="5">
+    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -3643,18 +3595,19 @@
       <c r="D3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="1">
         <v>1</v>
       </c>
-      <c r="F3" s="7">
-        <f>F2+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="5">
+      <c r="F3" s="1">
+        <f t="shared" ref="F3:F31" si="0">F2+1</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -3663,18 +3616,19 @@
       <c r="D4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="1">
         <v>1</v>
       </c>
-      <c r="F4" s="7">
-        <f>F3+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="5">
+      <c r="F4" s="1">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -3683,18 +3637,19 @@
       <c r="D5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="1">
         <v>1</v>
       </c>
-      <c r="F5" s="7">
-        <f>F4+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="5">
+      <c r="F5" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -3703,18 +3658,19 @@
       <c r="D6" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="1">
         <v>1</v>
       </c>
-      <c r="F6" s="7">
-        <f>F5+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="5">
+      <c r="F6" s="1">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -3723,18 +3679,19 @@
       <c r="D7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="1">
         <v>1</v>
       </c>
-      <c r="F7" s="7">
-        <f>F6+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="5">
+      <c r="F7" s="1">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -3743,18 +3700,19 @@
       <c r="D8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="1">
         <v>1</v>
       </c>
-      <c r="F8" s="7">
-        <f>F7+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="5">
+      <c r="F8" s="1">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -3763,18 +3721,19 @@
       <c r="D9" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="1">
         <v>1</v>
       </c>
-      <c r="F9" s="7">
-        <f>F8+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="5">
+      <c r="F9" s="1">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -3783,18 +3742,19 @@
       <c r="D10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="1">
         <v>1</v>
       </c>
-      <c r="F10" s="7">
-        <f>F9+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="5">
+      <c r="F10" s="1">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -3803,18 +3763,19 @@
       <c r="D11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="1">
         <v>1</v>
       </c>
-      <c r="F11" s="7">
-        <f>F10+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="5">
+      <c r="F11" s="1">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -3823,18 +3784,19 @@
       <c r="D12" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="1">
         <v>1</v>
       </c>
-      <c r="F12" s="7">
-        <f>F11+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="5">
-        <f>A12+1</f>
-      </c>
-      <c r="B13" s="6" t="s">
+      <c r="F12" s="1">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -3843,18 +3805,19 @@
       <c r="D13" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="1">
         <v>1</v>
       </c>
-      <c r="F13" s="7">
-        <f>F12+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="5">
-        <f>A13+1</f>
-      </c>
-      <c r="B14" s="6" t="s">
+      <c r="F13" s="1">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -3863,18 +3826,19 @@
       <c r="D14" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="1">
         <v>1</v>
       </c>
-      <c r="F14" s="7">
-        <f>F13+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="5">
-        <f>A14+1</f>
-      </c>
-      <c r="B15" s="6" t="s">
+      <c r="F14" s="1">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -3883,18 +3847,19 @@
       <c r="D15" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="1">
         <v>1</v>
       </c>
-      <c r="F15" s="7">
-        <f>F14+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="5">
-        <f>A15+1</f>
-      </c>
-      <c r="B16" s="6" t="s">
+      <c r="F15" s="1">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -3903,18 +3868,19 @@
       <c r="D16" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="1">
         <v>1</v>
       </c>
-      <c r="F16" s="7">
-        <f>F15+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="5">
-        <f>A16+1</f>
-      </c>
-      <c r="B17" s="6" t="s">
+      <c r="F16" s="1">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -3923,18 +3889,19 @@
       <c r="D17" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="1">
         <v>1</v>
       </c>
-      <c r="F17" s="7">
-        <f>F16+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="5">
-        <f>A17+1</f>
-      </c>
-      <c r="B18" s="6" t="s">
+      <c r="F17" s="1">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -3943,18 +3910,19 @@
       <c r="D18" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="1">
         <v>1</v>
       </c>
-      <c r="F18" s="7">
-        <f>F17+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="5">
-        <f>A18+1</f>
-      </c>
-      <c r="B19" s="6" t="s">
+      <c r="F18" s="1">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -3963,18 +3931,19 @@
       <c r="D19" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="1">
         <v>1</v>
       </c>
-      <c r="F19" s="7">
-        <f>F18+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="5">
-        <f>A19+1</f>
-      </c>
-      <c r="B20" s="6" t="s">
+      <c r="F19" s="1">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -3983,18 +3952,19 @@
       <c r="D20" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="1">
         <v>1</v>
       </c>
-      <c r="F20" s="7">
-        <f>F19+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="5">
-        <f>A20+1</f>
-      </c>
-      <c r="B21" s="6" t="s">
+      <c r="F20" s="1">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -4003,18 +3973,19 @@
       <c r="D21" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="1">
         <v>1</v>
       </c>
-      <c r="F21" s="7">
-        <f>F20+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="5">
-        <f>A21+1</f>
-      </c>
-      <c r="B22" s="6" t="s">
+      <c r="F21" s="1">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -4023,18 +3994,19 @@
       <c r="D22" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="1">
         <v>1</v>
       </c>
-      <c r="F22" s="7">
-        <f>F21+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="5">
-        <f>A22+1</f>
-      </c>
-      <c r="B23" s="6" t="s">
+      <c r="F22" s="1">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -4043,18 +4015,19 @@
       <c r="D23" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="1">
         <v>1</v>
       </c>
-      <c r="F23" s="7">
-        <f>F22+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="5">
-        <f>A23+1</f>
-      </c>
-      <c r="B24" s="6" t="s">
+      <c r="F23" s="1">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -4063,18 +4036,19 @@
       <c r="D24" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E24" s="5">
+      <c r="E24" s="1">
         <v>1</v>
       </c>
-      <c r="F24" s="7">
-        <f>F23+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="5">
-        <f>A24+1</f>
-      </c>
-      <c r="B25" s="6" t="s">
+      <c r="F24" s="1">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -4083,18 +4057,19 @@
       <c r="D25" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="5">
+      <c r="E25" s="1">
         <v>1</v>
       </c>
-      <c r="F25" s="7">
-        <f>F24+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="5">
-        <f>A25+1</f>
-      </c>
-      <c r="B26" s="6" t="s">
+      <c r="F25" s="1">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C26" s="2" t="s">
@@ -4103,18 +4078,19 @@
       <c r="D26" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E26" s="5">
+      <c r="E26" s="1">
         <v>1</v>
       </c>
-      <c r="F26" s="7">
-        <f>F25+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="5">
-        <f>A26+1</f>
-      </c>
-      <c r="B27" s="6" t="s">
+      <c r="F26" s="1">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C27" s="2" t="s">
@@ -4123,18 +4099,19 @@
       <c r="D27" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="5">
+      <c r="E27" s="1">
         <v>1</v>
       </c>
-      <c r="F27" s="7">
-        <f>F26+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
-      <c r="A28" s="5">
-        <f>A27+1</f>
-      </c>
-      <c r="B28" s="6" t="s">
+      <c r="F27" s="1">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="1">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -4143,18 +4120,19 @@
       <c r="D28" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E28" s="5">
+      <c r="E28" s="1">
         <v>1</v>
       </c>
-      <c r="F28" s="7">
-        <f>F27+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
-      <c r="A29" s="5">
-        <f>A28+1</f>
-      </c>
-      <c r="B29" s="6" t="s">
+      <c r="F28" s="1">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C29" s="2" t="s">
@@ -4163,18 +4141,19 @@
       <c r="D29" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="5">
+      <c r="E29" s="1">
         <v>1</v>
       </c>
-      <c r="F29" s="7">
-        <f>F28+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
-      <c r="A30" s="5">
-        <f>A29+1</f>
-      </c>
-      <c r="B30" s="6" t="s">
+      <c r="F29" s="1">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="1">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -4183,18 +4162,19 @@
       <c r="D30" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E30" s="5">
+      <c r="E30" s="1">
         <v>1</v>
       </c>
-      <c r="F30" s="7">
-        <f>F29+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
-      <c r="A31" s="5">
-        <f>A30+1</f>
-      </c>
-      <c r="B31" s="6" t="s">
+      <c r="F30" s="1">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C31" s="2" t="s">
@@ -4203,18 +4183,19 @@
       <c r="D31" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E31" s="5">
+      <c r="E31" s="1">
         <v>1</v>
       </c>
-      <c r="F31" s="7">
-        <f>F30+1</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="5">
+      <c r="F31" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="1">
         <v>31</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C32" s="2" t="s">
@@ -4226,13 +4207,13 @@
       <c r="E32" s="1">
         <v>0</v>
       </c>
-      <c r="F32" s="7">
+      <c r="F32" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="7">
-        <f>A32+1</f>
+    <row r="33" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
+        <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>5</v>
@@ -4243,16 +4224,16 @@
       <c r="D33" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E33" s="7">
-        <v>0</v>
-      </c>
-      <c r="F33" s="7">
+      <c r="E33" s="1">
+        <v>0</v>
+      </c>
+      <c r="F33" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="7">
-        <f>A33+1</f>
+    <row r="34" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
+        <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>5</v>
@@ -4263,16 +4244,16 @@
       <c r="D34" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E34" s="7">
-        <v>0</v>
-      </c>
-      <c r="F34" s="7">
+      <c r="E34" s="1">
+        <v>0</v>
+      </c>
+      <c r="F34" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
-      <c r="A35" s="7">
-        <f>A34+1</f>
+    <row r="35" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="1">
+        <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>5</v>
@@ -4283,16 +4264,16 @@
       <c r="D35" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E35" s="7">
-        <v>0</v>
-      </c>
-      <c r="F35" s="7">
+      <c r="E35" s="1">
+        <v>0</v>
+      </c>
+      <c r="F35" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="7">
-        <f>A35+1</f>
+    <row r="36" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
+        <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>5</v>
@@ -4303,16 +4284,16 @@
       <c r="D36" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E36" s="7">
-        <v>0</v>
-      </c>
-      <c r="F36" s="7">
+      <c r="E36" s="1">
+        <v>0</v>
+      </c>
+      <c r="F36" s="1">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="7">
-        <f>A36+1</f>
+    <row r="37" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="1">
+        <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>7</v>
@@ -4323,16 +4304,16 @@
       <c r="D37" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E37" s="7">
-        <v>0</v>
-      </c>
-      <c r="F37" s="7">
+      <c r="E37" s="1">
+        <v>0</v>
+      </c>
+      <c r="F37" s="1">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
-      <c r="A38" s="7">
-        <f>A37+1</f>
+    <row r="38" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="1">
+        <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>7</v>
@@ -4343,16 +4324,16 @@
       <c r="D38" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E38" s="7">
-        <v>0</v>
-      </c>
-      <c r="F38" s="7">
+      <c r="E38" s="1">
+        <v>0</v>
+      </c>
+      <c r="F38" s="1">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="7">
-        <f>A38+1</f>
+    <row r="39" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
+        <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>7</v>
@@ -4363,16 +4344,16 @@
       <c r="D39" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E39" s="7">
-        <v>0</v>
-      </c>
-      <c r="F39" s="7">
+      <c r="E39" s="1">
+        <v>0</v>
+      </c>
+      <c r="F39" s="1">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
-      <c r="A40" s="7">
-        <f>A39+1</f>
+    <row r="40" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
+        <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>7</v>
@@ -4383,16 +4364,16 @@
       <c r="D40" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E40" s="7">
-        <v>0</v>
-      </c>
-      <c r="F40" s="7">
+      <c r="E40" s="1">
+        <v>0</v>
+      </c>
+      <c r="F40" s="1">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
-      <c r="A41" s="7">
-        <f>A40+1</f>
+    <row r="41" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="1">
+        <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>9</v>
@@ -4403,16 +4384,16 @@
       <c r="D41" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E41" s="7">
-        <v>0</v>
-      </c>
-      <c r="F41" s="7">
+      <c r="E41" s="1">
+        <v>0</v>
+      </c>
+      <c r="F41" s="1">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
-      <c r="A42" s="7">
-        <f>A41+1</f>
+    <row r="42" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="1">
+        <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>9</v>
@@ -4423,16 +4404,16 @@
       <c r="D42" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E42" s="7">
-        <v>0</v>
-      </c>
-      <c r="F42" s="7">
+      <c r="E42" s="1">
+        <v>0</v>
+      </c>
+      <c r="F42" s="1">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
-      <c r="A43" s="7">
-        <f>A42+1</f>
+    <row r="43" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="1">
+        <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>9</v>
@@ -4443,16 +4424,16 @@
       <c r="D43" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E43" s="7">
-        <v>0</v>
-      </c>
-      <c r="F43" s="7">
+      <c r="E43" s="1">
+        <v>0</v>
+      </c>
+      <c r="F43" s="1">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
-      <c r="A44" s="7">
-        <f>A43+1</f>
+    <row r="44" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="1">
+        <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>5</v>
@@ -4463,16 +4444,16 @@
       <c r="D44" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E44" s="7">
-        <v>0</v>
-      </c>
-      <c r="F44" s="7">
+      <c r="E44" s="1">
+        <v>0</v>
+      </c>
+      <c r="F44" s="1">
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
-      <c r="A45" s="7">
-        <f>A44+1</f>
+    <row r="45" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="1">
+        <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>5</v>
@@ -4483,16 +4464,16 @@
       <c r="D45" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E45" s="7">
-        <v>0</v>
-      </c>
-      <c r="F45" s="7">
+      <c r="E45" s="1">
+        <v>0</v>
+      </c>
+      <c r="F45" s="1">
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
-      <c r="A46" s="7">
-        <f>A45+1</f>
+    <row r="46" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="1">
+        <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>5</v>
@@ -4503,16 +4484,16 @@
       <c r="D46" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E46" s="7">
-        <v>0</v>
-      </c>
-      <c r="F46" s="7">
+      <c r="E46" s="1">
+        <v>0</v>
+      </c>
+      <c r="F46" s="1">
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
-      <c r="A47" s="7">
-        <f>A46+1</f>
+    <row r="47" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="1">
+        <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>7</v>
@@ -4523,16 +4504,16 @@
       <c r="D47" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E47" s="7">
-        <v>0</v>
-      </c>
-      <c r="F47" s="7">
+      <c r="E47" s="1">
+        <v>0</v>
+      </c>
+      <c r="F47" s="1">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
-      <c r="A48" s="7">
-        <f>A47+1</f>
+    <row r="48" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="1">
+        <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>7</v>
@@ -4543,16 +4524,16 @@
       <c r="D48" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E48" s="7">
-        <v>0</v>
-      </c>
-      <c r="F48" s="7">
+      <c r="E48" s="1">
+        <v>0</v>
+      </c>
+      <c r="F48" s="1">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
-      <c r="A49" s="7">
-        <f>A48+1</f>
+    <row r="49" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="1">
+        <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>7</v>
@@ -4563,16 +4544,16 @@
       <c r="D49" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E49" s="7">
-        <v>0</v>
-      </c>
-      <c r="F49" s="7">
+      <c r="E49" s="1">
+        <v>0</v>
+      </c>
+      <c r="F49" s="1">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
-      <c r="A50" s="7">
-        <f>A49+1</f>
+    <row r="50" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="1">
+        <v>49</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>9</v>
@@ -4583,16 +4564,16 @@
       <c r="D50" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E50" s="7">
-        <v>0</v>
-      </c>
-      <c r="F50" s="7">
+      <c r="E50" s="1">
+        <v>0</v>
+      </c>
+      <c r="F50" s="1">
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
-      <c r="A51" s="7">
-        <f>A50+1</f>
+    <row r="51" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="1">
+        <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>9</v>
@@ -4603,16 +4584,16 @@
       <c r="D51" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E51" s="7">
-        <v>0</v>
-      </c>
-      <c r="F51" s="7">
+      <c r="E51" s="1">
+        <v>0</v>
+      </c>
+      <c r="F51" s="1">
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
-      <c r="A52" s="7">
-        <f>A51+1</f>
+    <row r="52" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="1">
+        <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>9</v>
@@ -4623,16 +4604,16 @@
       <c r="D52" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E52" s="7">
-        <v>0</v>
-      </c>
-      <c r="F52" s="7">
+      <c r="E52" s="1">
+        <v>0</v>
+      </c>
+      <c r="F52" s="1">
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
-      <c r="A53" s="7">
-        <f>A52+1</f>
+    <row r="53" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="1">
+        <v>52</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>5</v>
@@ -4643,16 +4624,16 @@
       <c r="D53" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E53" s="7">
-        <v>0</v>
-      </c>
-      <c r="F53" s="7">
+      <c r="E53" s="1">
+        <v>0</v>
+      </c>
+      <c r="F53" s="1">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
-      <c r="A54" s="7">
-        <f>A53+1</f>
+    <row r="54" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="1">
+        <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>5</v>
@@ -4663,16 +4644,16 @@
       <c r="D54" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E54" s="7">
-        <v>0</v>
-      </c>
-      <c r="F54" s="7">
+      <c r="E54" s="1">
+        <v>0</v>
+      </c>
+      <c r="F54" s="1">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
-      <c r="A55" s="7">
-        <f>A54+1</f>
+    <row r="55" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="1">
+        <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>5</v>
@@ -4683,16 +4664,16 @@
       <c r="D55" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E55" s="7">
-        <v>0</v>
-      </c>
-      <c r="F55" s="7">
+      <c r="E55" s="1">
+        <v>0</v>
+      </c>
+      <c r="F55" s="1">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
-      <c r="A56" s="7">
-        <f>A55+1</f>
+    <row r="56" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="1">
+        <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>5</v>
@@ -4703,16 +4684,16 @@
       <c r="D56" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E56" s="7">
-        <v>0</v>
-      </c>
-      <c r="F56" s="7">
+      <c r="E56" s="1">
+        <v>0</v>
+      </c>
+      <c r="F56" s="1">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
-      <c r="A57" s="7">
-        <f>A56+1</f>
+    <row r="57" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="1">
+        <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>5</v>
@@ -4723,16 +4704,16 @@
       <c r="D57" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E57" s="7">
-        <v>0</v>
-      </c>
-      <c r="F57" s="7">
+      <c r="E57" s="1">
+        <v>0</v>
+      </c>
+      <c r="F57" s="1">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
-      <c r="A58" s="7">
-        <f>A57+1</f>
+    <row r="58" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="1">
+        <v>57</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>7</v>
@@ -4743,16 +4724,16 @@
       <c r="D58" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E58" s="7">
-        <v>0</v>
-      </c>
-      <c r="F58" s="7">
+      <c r="E58" s="1">
+        <v>0</v>
+      </c>
+      <c r="F58" s="1">
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
-      <c r="A59" s="7">
-        <f>A58+1</f>
+    <row r="59" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="1">
+        <v>58</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>7</v>
@@ -4763,16 +4744,16 @@
       <c r="D59" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E59" s="7">
-        <v>0</v>
-      </c>
-      <c r="F59" s="7">
+      <c r="E59" s="1">
+        <v>0</v>
+      </c>
+      <c r="F59" s="1">
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
-      <c r="A60" s="7">
-        <f>A59+1</f>
+    <row r="60" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="1">
+        <v>59</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>7</v>
@@ -4783,16 +4764,16 @@
       <c r="D60" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E60" s="7">
-        <v>0</v>
-      </c>
-      <c r="F60" s="7">
+      <c r="E60" s="1">
+        <v>0</v>
+      </c>
+      <c r="F60" s="1">
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
-      <c r="A61" s="7">
-        <f>A60+1</f>
+    <row r="61" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="1">
+        <v>60</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>9</v>
@@ -4803,16 +4784,16 @@
       <c r="D61" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E61" s="7">
-        <v>0</v>
-      </c>
-      <c r="F61" s="7">
+      <c r="E61" s="1">
+        <v>0</v>
+      </c>
+      <c r="F61" s="1">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
-      <c r="A62" s="7">
-        <f>A61+1</f>
+    <row r="62" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="1">
+        <v>61</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>9</v>
@@ -4823,16 +4804,16 @@
       <c r="D62" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E62" s="7">
-        <v>0</v>
-      </c>
-      <c r="F62" s="7">
+      <c r="E62" s="1">
+        <v>0</v>
+      </c>
+      <c r="F62" s="1">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
-      <c r="A63" s="7">
-        <f>A62+1</f>
+    <row r="63" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="1">
+        <v>62</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>9</v>
@@ -4843,16 +4824,16 @@
       <c r="D63" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E63" s="7">
-        <v>0</v>
-      </c>
-      <c r="F63" s="7">
+      <c r="E63" s="1">
+        <v>0</v>
+      </c>
+      <c r="F63" s="1">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
-      <c r="A64" s="7">
-        <f>A63+1</f>
+    <row r="64" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="1">
+        <v>63</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>5</v>
@@ -4863,16 +4844,16 @@
       <c r="D64" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E64" s="7">
-        <v>0</v>
-      </c>
-      <c r="F64" s="7">
+      <c r="E64" s="1">
+        <v>0</v>
+      </c>
+      <c r="F64" s="1">
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
-      <c r="A65" s="7">
-        <f>A64+1</f>
+    <row r="65" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="1">
+        <v>64</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>5</v>
@@ -4883,16 +4864,16 @@
       <c r="D65" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E65" s="7">
-        <v>0</v>
-      </c>
-      <c r="F65" s="7">
+      <c r="E65" s="1">
+        <v>0</v>
+      </c>
+      <c r="F65" s="1">
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
-      <c r="A66" s="7">
-        <f>A65+1</f>
+    <row r="66" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="1">
+        <v>65</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>5</v>
@@ -4903,16 +4884,16 @@
       <c r="D66" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E66" s="7">
-        <v>0</v>
-      </c>
-      <c r="F66" s="7">
+      <c r="E66" s="1">
+        <v>0</v>
+      </c>
+      <c r="F66" s="1">
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
-      <c r="A67" s="7">
-        <f>A66+1</f>
+    <row r="67" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="1">
+        <v>66</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>7</v>
@@ -4923,16 +4904,16 @@
       <c r="D67" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E67" s="7">
-        <v>0</v>
-      </c>
-      <c r="F67" s="7">
+      <c r="E67" s="1">
+        <v>0</v>
+      </c>
+      <c r="F67" s="1">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
-      <c r="A68" s="7">
-        <f>A67+1</f>
+    <row r="68" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="1">
+        <v>67</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>7</v>
@@ -4943,16 +4924,16 @@
       <c r="D68" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E68" s="7">
-        <v>0</v>
-      </c>
-      <c r="F68" s="7">
+      <c r="E68" s="1">
+        <v>0</v>
+      </c>
+      <c r="F68" s="1">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
-      <c r="A69" s="7">
-        <f>A68+1</f>
+    <row r="69" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="1">
+        <v>68</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>7</v>
@@ -4963,16 +4944,16 @@
       <c r="D69" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E69" s="7">
-        <v>0</v>
-      </c>
-      <c r="F69" s="7">
+      <c r="E69" s="1">
+        <v>0</v>
+      </c>
+      <c r="F69" s="1">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
-      <c r="A70" s="7">
-        <f>A69+1</f>
+    <row r="70" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="1">
+        <v>69</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>7</v>
@@ -4983,16 +4964,16 @@
       <c r="D70" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E70" s="7">
-        <v>0</v>
-      </c>
-      <c r="F70" s="7">
+      <c r="E70" s="1">
+        <v>0</v>
+      </c>
+      <c r="F70" s="1">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
-      <c r="A71" s="7">
-        <f>A70+1</f>
+    <row r="71" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="1">
+        <v>70</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>7</v>
@@ -5003,16 +4984,16 @@
       <c r="D71" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E71" s="7">
-        <v>0</v>
-      </c>
-      <c r="F71" s="7">
+      <c r="E71" s="1">
+        <v>0</v>
+      </c>
+      <c r="F71" s="1">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
-      <c r="A72" s="7">
-        <f>A71+1</f>
+    <row r="72" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="1">
+        <v>71</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>9</v>
@@ -5023,16 +5004,16 @@
       <c r="D72" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E72" s="7">
-        <v>0</v>
-      </c>
-      <c r="F72" s="7">
+      <c r="E72" s="1">
+        <v>0</v>
+      </c>
+      <c r="F72" s="1">
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
-      <c r="A73" s="7">
-        <f>A72+1</f>
+    <row r="73" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="1">
+        <v>72</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>9</v>
@@ -5043,16 +5024,16 @@
       <c r="D73" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E73" s="7">
-        <v>0</v>
-      </c>
-      <c r="F73" s="7">
+      <c r="E73" s="1">
+        <v>0</v>
+      </c>
+      <c r="F73" s="1">
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
-      <c r="A74" s="7">
-        <f>A73+1</f>
+    <row r="74" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="1">
+        <v>73</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>9</v>
@@ -5063,336 +5044,342 @@
       <c r="D74" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E74" s="7">
-        <v>0</v>
-      </c>
-      <c r="F74" s="7">
+      <c r="E74" s="1">
+        <v>0</v>
+      </c>
+      <c r="F74" s="1">
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
-      <c r="A75" s="7">
-        <f>A74+1</f>
-      </c>
-      <c r="B75" s="8"/>
-      <c r="C75" s="8"/>
-      <c r="D75" s="8"/>
-      <c r="E75" s="7">
-        <v>0</v>
-      </c>
-      <c r="F75" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
-      <c r="A76" s="7">
-        <f>A75+1</f>
-      </c>
-      <c r="B76" s="8"/>
-      <c r="C76" s="8"/>
-      <c r="D76" s="8"/>
-      <c r="E76" s="7">
-        <v>0</v>
-      </c>
-      <c r="F76" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
-      <c r="A77" s="7">
-        <f>A76+1</f>
-      </c>
-      <c r="B77" s="8"/>
-      <c r="C77" s="8"/>
-      <c r="D77" s="8"/>
-      <c r="E77" s="7">
-        <v>0</v>
-      </c>
-      <c r="F77" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
-      <c r="A78" s="7">
-        <f>A77+1</f>
-      </c>
-      <c r="B78" s="8"/>
-      <c r="C78" s="8"/>
-      <c r="D78" s="8"/>
-      <c r="E78" s="7">
-        <v>0</v>
-      </c>
-      <c r="F78" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
-      <c r="A79" s="7">
-        <f>A78+1</f>
-      </c>
-      <c r="B79" s="8"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="8"/>
-      <c r="E79" s="7">
-        <v>0</v>
-      </c>
-      <c r="F79" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
-      <c r="A80" s="7">
-        <f>A79+1</f>
-      </c>
-      <c r="B80" s="8"/>
-      <c r="C80" s="8"/>
-      <c r="D80" s="8"/>
-      <c r="E80" s="7">
-        <v>0</v>
-      </c>
-      <c r="F80" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
-      <c r="A81" s="7">
-        <f>A80+1</f>
-      </c>
-      <c r="B81" s="8"/>
-      <c r="C81" s="8"/>
-      <c r="D81" s="8"/>
-      <c r="E81" s="7">
-        <v>0</v>
-      </c>
-      <c r="F81" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
-      <c r="A82" s="7">
-        <f>A81+1</f>
-      </c>
-      <c r="B82" s="8"/>
-      <c r="C82" s="8"/>
-      <c r="D82" s="8"/>
-      <c r="E82" s="7">
-        <v>0</v>
-      </c>
-      <c r="F82" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
-      <c r="A83" s="7">
-        <f>A82+1</f>
-      </c>
-      <c r="B83" s="8"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="8"/>
-      <c r="E83" s="7">
-        <v>0</v>
-      </c>
-      <c r="F83" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
-      <c r="A84" s="7">
-        <f>A83+1</f>
-      </c>
-      <c r="B84" s="8"/>
-      <c r="C84" s="8"/>
-      <c r="D84" s="8"/>
-      <c r="E84" s="7">
-        <v>0</v>
-      </c>
-      <c r="F84" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
-      <c r="A85" s="7">
-        <f>A84+1</f>
-      </c>
-      <c r="B85" s="8"/>
-      <c r="C85" s="8"/>
-      <c r="D85" s="8"/>
-      <c r="E85" s="7">
-        <v>0</v>
-      </c>
-      <c r="F85" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
-      <c r="A86" s="7">
-        <f>A85+1</f>
-      </c>
-      <c r="B86" s="8"/>
-      <c r="C86" s="8"/>
-      <c r="D86" s="8"/>
-      <c r="E86" s="7">
-        <v>0</v>
-      </c>
-      <c r="F86" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
-      <c r="A87" s="7">
-        <f>A86+1</f>
-      </c>
-      <c r="B87" s="8"/>
-      <c r="C87" s="8"/>
-      <c r="D87" s="8"/>
-      <c r="E87" s="7">
-        <v>0</v>
-      </c>
-      <c r="F87" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
-      <c r="A88" s="7">
-        <f>A87+1</f>
-      </c>
-      <c r="B88" s="8"/>
-      <c r="C88" s="8"/>
-      <c r="D88" s="8"/>
-      <c r="E88" s="7">
-        <v>0</v>
-      </c>
-      <c r="F88" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
-      <c r="A89" s="7">
-        <f>A88+1</f>
-      </c>
-      <c r="B89" s="8"/>
-      <c r="C89" s="8"/>
-      <c r="D89" s="8"/>
-      <c r="E89" s="7">
-        <v>0</v>
-      </c>
-      <c r="F89" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
-      <c r="A90" s="7">
-        <f>A89+1</f>
-      </c>
-      <c r="B90" s="8"/>
-      <c r="C90" s="8"/>
-      <c r="D90" s="8"/>
-      <c r="E90" s="7">
-        <v>0</v>
-      </c>
-      <c r="F90" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
-      <c r="A91" s="7">
-        <f>A90+1</f>
-      </c>
-      <c r="B91" s="8"/>
-      <c r="C91" s="8"/>
-      <c r="D91" s="8"/>
-      <c r="E91" s="7">
-        <v>0</v>
-      </c>
-      <c r="F91" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
-      <c r="A92" s="7">
-        <f>A91+1</f>
-      </c>
-      <c r="B92" s="8"/>
-      <c r="C92" s="8"/>
-      <c r="D92" s="8"/>
-      <c r="E92" s="7">
-        <v>0</v>
-      </c>
-      <c r="F92" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
-      <c r="A93" s="7">
-        <f>A92+1</f>
-      </c>
-      <c r="B93" s="8"/>
-      <c r="C93" s="8"/>
-      <c r="D93" s="8"/>
-      <c r="E93" s="7">
-        <v>0</v>
-      </c>
-      <c r="F93" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
-      <c r="A94" s="7">
-        <f>A93+1</f>
-      </c>
-      <c r="B94" s="8"/>
-      <c r="C94" s="8"/>
-      <c r="D94" s="8"/>
-      <c r="E94" s="7">
-        <v>0</v>
-      </c>
-      <c r="F94" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
-      <c r="A95" s="7">
-        <f>A94+1</f>
-      </c>
-      <c r="B95" s="8"/>
-      <c r="C95" s="8"/>
-      <c r="D95" s="8"/>
-      <c r="E95" s="7">
-        <v>0</v>
-      </c>
-      <c r="F95" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
-      <c r="A96" s="7">
-        <f>A95+1</f>
-      </c>
-      <c r="B96" s="8"/>
-      <c r="C96" s="8"/>
-      <c r="D96" s="8"/>
-      <c r="E96" s="7">
-        <v>0</v>
-      </c>
-      <c r="F96" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
-      <c r="A97" s="7">
-        <f>A96+1</f>
-      </c>
-      <c r="B97" s="8"/>
-      <c r="C97" s="8"/>
-      <c r="D97" s="8"/>
-      <c r="E97" s="7">
-        <v>0</v>
-      </c>
-      <c r="F97" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
-      <c r="A98" s="7">
-        <f>A97+1</f>
-      </c>
-      <c r="B98" s="8"/>
-      <c r="C98" s="8"/>
-      <c r="D98" s="8"/>
-      <c r="E98" s="7">
-        <v>0</v>
-      </c>
-      <c r="F98" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
-      <c r="A99" s="7">
-        <f>A98+1</f>
-      </c>
-      <c r="B99" s="8"/>
-      <c r="C99" s="8"/>
-      <c r="D99" s="8"/>
-      <c r="E99" s="7">
-        <v>0</v>
-      </c>
-      <c r="F99" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
-      <c r="A100" s="7">
-        <f>A99+1</f>
-      </c>
-      <c r="B100" s="8"/>
-      <c r="C100" s="8"/>
-      <c r="D100" s="8"/>
-      <c r="E100" s="7">
-        <v>0</v>
-      </c>
-      <c r="F100" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
-      <c r="A101" s="7">
-        <f>A100+1</f>
-      </c>
-      <c r="B101" s="8"/>
-      <c r="C101" s="8"/>
-      <c r="D101" s="8"/>
-      <c r="E101" s="7">
-        <v>0</v>
-      </c>
-      <c r="F101" s="9"/>
+    <row r="75" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="1">
+        <v>74</v>
+      </c>
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="1">
+        <v>0</v>
+      </c>
+      <c r="F75" s="10"/>
+    </row>
+    <row r="76" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="1">
+        <v>75</v>
+      </c>
+      <c r="B76" s="4"/>
+      <c r="C76" s="4"/>
+      <c r="D76" s="4"/>
+      <c r="E76" s="1">
+        <v>0</v>
+      </c>
+      <c r="F76" s="10"/>
+    </row>
+    <row r="77" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="1">
+        <v>76</v>
+      </c>
+      <c r="B77" s="4"/>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="1">
+        <v>0</v>
+      </c>
+      <c r="F77" s="10"/>
+    </row>
+    <row r="78" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="1">
+        <v>77</v>
+      </c>
+      <c r="B78" s="4"/>
+      <c r="C78" s="4"/>
+      <c r="D78" s="4"/>
+      <c r="E78" s="1">
+        <v>0</v>
+      </c>
+      <c r="F78" s="10"/>
+    </row>
+    <row r="79" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="1">
+        <v>78</v>
+      </c>
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="4"/>
+      <c r="E79" s="1">
+        <v>0</v>
+      </c>
+      <c r="F79" s="10"/>
+    </row>
+    <row r="80" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="1">
+        <v>79</v>
+      </c>
+      <c r="B80" s="4"/>
+      <c r="C80" s="4"/>
+      <c r="D80" s="4"/>
+      <c r="E80" s="1">
+        <v>0</v>
+      </c>
+      <c r="F80" s="10"/>
+    </row>
+    <row r="81" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="1">
+        <v>80</v>
+      </c>
+      <c r="B81" s="4"/>
+      <c r="C81" s="4"/>
+      <c r="D81" s="4"/>
+      <c r="E81" s="1">
+        <v>0</v>
+      </c>
+      <c r="F81" s="10"/>
+    </row>
+    <row r="82" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="1">
+        <v>81</v>
+      </c>
+      <c r="B82" s="4"/>
+      <c r="C82" s="4"/>
+      <c r="D82" s="4"/>
+      <c r="E82" s="1">
+        <v>0</v>
+      </c>
+      <c r="F82" s="10"/>
+    </row>
+    <row r="83" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="1">
+        <v>82</v>
+      </c>
+      <c r="B83" s="4"/>
+      <c r="C83" s="4"/>
+      <c r="D83" s="4"/>
+      <c r="E83" s="1">
+        <v>0</v>
+      </c>
+      <c r="F83" s="10"/>
+    </row>
+    <row r="84" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="1">
+        <v>83</v>
+      </c>
+      <c r="B84" s="4"/>
+      <c r="C84" s="4"/>
+      <c r="D84" s="4"/>
+      <c r="E84" s="1">
+        <v>0</v>
+      </c>
+      <c r="F84" s="10"/>
+    </row>
+    <row r="85" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="1">
+        <v>84</v>
+      </c>
+      <c r="B85" s="4"/>
+      <c r="C85" s="4"/>
+      <c r="D85" s="4"/>
+      <c r="E85" s="1">
+        <v>0</v>
+      </c>
+      <c r="F85" s="10"/>
+    </row>
+    <row r="86" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="1">
+        <v>85</v>
+      </c>
+      <c r="B86" s="4"/>
+      <c r="C86" s="4"/>
+      <c r="D86" s="4"/>
+      <c r="E86" s="1">
+        <v>0</v>
+      </c>
+      <c r="F86" s="10"/>
+    </row>
+    <row r="87" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="1">
+        <v>86</v>
+      </c>
+      <c r="B87" s="4"/>
+      <c r="C87" s="4"/>
+      <c r="D87" s="4"/>
+      <c r="E87" s="1">
+        <v>0</v>
+      </c>
+      <c r="F87" s="10"/>
+    </row>
+    <row r="88" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="1">
+        <v>87</v>
+      </c>
+      <c r="B88" s="4"/>
+      <c r="C88" s="4"/>
+      <c r="D88" s="4"/>
+      <c r="E88" s="1">
+        <v>0</v>
+      </c>
+      <c r="F88" s="10"/>
+    </row>
+    <row r="89" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="1">
+        <v>88</v>
+      </c>
+      <c r="B89" s="4"/>
+      <c r="C89" s="4"/>
+      <c r="D89" s="4"/>
+      <c r="E89" s="1">
+        <v>0</v>
+      </c>
+      <c r="F89" s="10"/>
+    </row>
+    <row r="90" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="1">
+        <v>89</v>
+      </c>
+      <c r="B90" s="4"/>
+      <c r="C90" s="4"/>
+      <c r="D90" s="4"/>
+      <c r="E90" s="1">
+        <v>0</v>
+      </c>
+      <c r="F90" s="10"/>
+    </row>
+    <row r="91" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="1">
+        <v>90</v>
+      </c>
+      <c r="B91" s="4"/>
+      <c r="C91" s="4"/>
+      <c r="D91" s="4"/>
+      <c r="E91" s="1">
+        <v>0</v>
+      </c>
+      <c r="F91" s="10"/>
+    </row>
+    <row r="92" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A92" s="1">
+        <v>91</v>
+      </c>
+      <c r="B92" s="4"/>
+      <c r="C92" s="4"/>
+      <c r="D92" s="4"/>
+      <c r="E92" s="1">
+        <v>0</v>
+      </c>
+      <c r="F92" s="10"/>
+    </row>
+    <row r="93" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A93" s="1">
+        <v>92</v>
+      </c>
+      <c r="B93" s="4"/>
+      <c r="C93" s="4"/>
+      <c r="D93" s="4"/>
+      <c r="E93" s="1">
+        <v>0</v>
+      </c>
+      <c r="F93" s="10"/>
+    </row>
+    <row r="94" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A94" s="1">
+        <v>93</v>
+      </c>
+      <c r="B94" s="4"/>
+      <c r="C94" s="4"/>
+      <c r="D94" s="4"/>
+      <c r="E94" s="1">
+        <v>0</v>
+      </c>
+      <c r="F94" s="10"/>
+    </row>
+    <row r="95" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A95" s="1">
+        <v>94</v>
+      </c>
+      <c r="B95" s="4"/>
+      <c r="C95" s="4"/>
+      <c r="D95" s="4"/>
+      <c r="E95" s="1">
+        <v>0</v>
+      </c>
+      <c r="F95" s="10"/>
+    </row>
+    <row r="96" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A96" s="1">
+        <v>95</v>
+      </c>
+      <c r="B96" s="4"/>
+      <c r="C96" s="4"/>
+      <c r="D96" s="4"/>
+      <c r="E96" s="1">
+        <v>0</v>
+      </c>
+      <c r="F96" s="10"/>
+    </row>
+    <row r="97" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A97" s="1">
+        <v>96</v>
+      </c>
+      <c r="B97" s="4"/>
+      <c r="C97" s="4"/>
+      <c r="D97" s="4"/>
+      <c r="E97" s="1">
+        <v>0</v>
+      </c>
+      <c r="F97" s="10"/>
+    </row>
+    <row r="98" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A98" s="1">
+        <v>97</v>
+      </c>
+      <c r="B98" s="4"/>
+      <c r="C98" s="4"/>
+      <c r="D98" s="4"/>
+      <c r="E98" s="1">
+        <v>0</v>
+      </c>
+      <c r="F98" s="10"/>
+    </row>
+    <row r="99" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A99" s="1">
+        <v>98</v>
+      </c>
+      <c r="B99" s="4"/>
+      <c r="C99" s="4"/>
+      <c r="D99" s="4"/>
+      <c r="E99" s="1">
+        <v>0</v>
+      </c>
+      <c r="F99" s="10"/>
+    </row>
+    <row r="100" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A100" s="1">
+        <v>99</v>
+      </c>
+      <c r="B100" s="4"/>
+      <c r="C100" s="4"/>
+      <c r="D100" s="4"/>
+      <c r="E100" s="1">
+        <v>0</v>
+      </c>
+      <c r="F100" s="10"/>
+    </row>
+    <row r="101" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A101" s="1">
+        <v>100</v>
+      </c>
+      <c r="B101" s="4"/>
+      <c r="C101" s="4"/>
+      <c r="D101" s="4"/>
+      <c r="E101" s="1">
+        <v>0</v>
+      </c>
+      <c r="F101" s="10"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A102" s="1">
+        <f t="shared" ref="A66:A102" si="1">A101+1</f>
+        <v>101</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5400,27 +5387,22 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:K31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="53.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="46.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="11" width="13.5" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5443,7 +5425,7 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -5466,7 +5448,7 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -5489,7 +5471,7 @@
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -5512,7 +5494,7 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -5535,7 +5517,7 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -5558,7 +5540,7 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -5581,7 +5563,7 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -5604,7 +5586,7 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row r="9" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -5627,7 +5609,7 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row r="10" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -5650,7 +5632,7 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row r="11" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -5673,7 +5655,7 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row r="12" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -5696,9 +5678,10 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row r="13" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
-        <f>A12+1</f>
+        <f t="shared" ref="A13:A31" si="0">A12+1</f>
+        <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>9</v>
@@ -5719,9 +5702,10 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row r="14" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <f>A13+1</f>
+        <f t="shared" si="0"/>
+        <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>5</v>
@@ -5742,9 +5726,10 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row r="15" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <f>A14+1</f>
+        <f t="shared" si="0"/>
+        <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>7</v>
@@ -5765,9 +5750,10 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row r="16" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
-        <f>A15+1</f>
+        <f t="shared" si="0"/>
+        <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>9</v>
@@ -5788,9 +5774,10 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row r="17" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
-        <f>A16+1</f>
+        <f t="shared" si="0"/>
+        <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>5</v>
@@ -5811,9 +5798,10 @@
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row r="18" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
-        <f>A17+1</f>
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>7</v>
@@ -5834,9 +5822,10 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row r="19" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <f>A18+1</f>
+        <f t="shared" si="0"/>
+        <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>9</v>
@@ -5857,9 +5846,10 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row r="20" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
-        <f>A19+1</f>
+        <f t="shared" si="0"/>
+        <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>5</v>
@@ -5880,9 +5870,10 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row r="21" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
-        <f>A20+1</f>
+        <f t="shared" si="0"/>
+        <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>7</v>
@@ -5903,9 +5894,10 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+    <row r="22" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
-        <f>A21+1</f>
+        <f t="shared" si="0"/>
+        <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>9</v>
@@ -5926,9 +5918,10 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+    <row r="23" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
-        <f>A22+1</f>
+        <f t="shared" si="0"/>
+        <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>5</v>
@@ -5949,9 +5942,10 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+    <row r="24" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
-        <f>A23+1</f>
+        <f t="shared" si="0"/>
+        <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>7</v>
@@ -5972,9 +5966,10 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+    <row r="25" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
-        <f>A24+1</f>
+        <f t="shared" si="0"/>
+        <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>9</v>
@@ -5995,9 +5990,10 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+    <row r="26" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
-        <f>A25+1</f>
+        <f t="shared" si="0"/>
+        <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>5</v>
@@ -6018,9 +6014,10 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+    <row r="27" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
-        <f>A26+1</f>
+        <f t="shared" si="0"/>
+        <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>7</v>
@@ -6041,9 +6038,10 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+    <row r="28" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
-        <f>A27+1</f>
+        <f t="shared" si="0"/>
+        <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>9</v>
@@ -6064,9 +6062,10 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+    <row r="29" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
-        <f>A28+1</f>
+        <f t="shared" si="0"/>
+        <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>5</v>
@@ -6087,9 +6086,10 @@
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+    <row r="30" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
-        <f>A29+1</f>
+        <f t="shared" si="0"/>
+        <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>7</v>
@@ -6110,9 +6110,10 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+    <row r="31" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
-        <f>A30+1</f>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>9</v>
@@ -6139,12 +6140,12 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>